<commit_message>
Cambios del 07-15 Abril
</commit_message>
<xml_diff>
--- a/PLANTILLAS MAIL/pruebas mail plantillas/base de plantilla.xlsx
+++ b/PLANTILLAS MAIL/pruebas mail plantillas/base de plantilla.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Explotación Phoenix\OneDrive - Phoenix Service\Escritorio\PROGRAMA\Formato_SMS\PLANTILLAS MAIL\pruebas mail plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://phoenixservice1-my.sharepoint.com/personal/fmontecino_phoenixservice_cl/Documents/Escritorio/PROGRAMA/Formato_SMS/PLANTILLAS MAIL/pruebas mail plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577744B4-497D-4496-A2AC-524F5E7C2A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{577744B4-497D-4496-A2AC-524F5E7C2A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B4338E6-77C7-4E2D-BFDA-C213650CD623}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>RUT</t>
   </si>
@@ -39,18 +39,9 @@
     <t>AGENTE</t>
   </si>
   <si>
-    <t>FONO AGENTE</t>
-  </si>
-  <si>
-    <t>MAIL AGENTE</t>
-  </si>
-  <si>
     <t>PIPE5550@GMAIL.COM</t>
   </si>
   <si>
-    <t>mperez@phlegal.cl</t>
-  </si>
-  <si>
     <t>Ariel Silva</t>
   </si>
   <si>
@@ -58,9 +49,6 @@
   </si>
   <si>
     <t>DV</t>
-  </si>
-  <si>
-    <t>asilva@phlegal.cl</t>
   </si>
 </sst>
 </file>
@@ -389,24 +377,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -417,14 +403,8 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>19361998</v>
       </c>
@@ -435,19 +415,13 @@
         <v>1234567890</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2">
-        <v>98789879</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>19361993</v>
       </c>
@@ -458,24 +432,16 @@
         <v>1234567890</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3">
-        <v>98789879</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{2CAC244E-747F-4DC6-8F8F-FDBB894A5B8A}"/>
-    <hyperlink ref="G2" r:id="rId2" xr:uid="{CD3F870B-4101-4756-AE36-827220330983}"/>
-    <hyperlink ref="D3" r:id="rId3" xr:uid="{4A3BD8BC-7E10-41BE-80B0-A4AC8E2C3541}"/>
-    <hyperlink ref="G3" r:id="rId4" xr:uid="{3AF222F9-BC08-47A7-9F72-AA2C46D64735}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{4A3BD8BC-7E10-41BE-80B0-A4AC8E2C3541}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>